<commit_message>
feat: update Ansible playbook summaries and consolidated files
</commit_message>
<xml_diff>
--- a/Ansible to Orchestrator Transition/Ansible_Playbook_Summaries.xlsx
+++ b/Ansible to Orchestrator Transition/Ansible_Playbook_Summaries.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Playbook Summaries" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Playbook Summaries'!$A$1:$C$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Playbook Summaries'!$A$1:$C$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,10 +480,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
@@ -629,7 +629,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Yes — Roles: roles/eam/, roles/envoy/, roles/lookup/, roles/perfcharts/, roles/postgresql/, roles/sts/, roles/ui/, roles/vami/, roles/vmware-photon-3.0-stig-ansible-hardening/, roles/vmware-photon-4.0-stig-ansible-hardening/, roles/vmware-photon-5.0-stig-ansible-hardening/</t>
+          <t>Yes — Roles: roles/eam/, roles/envoy/, roles/lookup/, roles/perfcharts/, roles/postgresql/, roles/sts/, roles/ui/, roles/vami/, roles/vmware-photon-{3,4,5}.0-stig-ansible-hardening/</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Windows Server security hardening for iPost remediation: disables SSL 2.0/3.0 and TLS 1.0/1.1 while enabling TLS 1.2/1.3 via registry, configures Memory Management speculative-execution mitigations, and enforces Network Level Authentication (NLA) for RDP.</t>
+          <t>Windows Server security hardening for iPost remediation: disables SSL 2.0/3.0 and TLS 1.0/1.1 while enabling TLS 1.2/1.3 via registry, configures Memory Management speculative-execution mitigations, and enforces NLA for RDP.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -668,666 +668,1084 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Microsoft Defender for Endpoint (MDE)</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ansible_post_stig.yml</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Applies the ansible_post_stig role to remediate or verify post-STIG configuration items on all targeted hosts.</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Role: roles/ansible_post_stig/</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>mde_gcc_install.yml</t>
+          <t>esxi-stig.yml</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Installs Microsoft Defender for Endpoint on RHEL (GCC environment variant). Installs yum-utils, stops fapolicyd if present, copies the GCC onboarding script, runs the Python onboarding, restarts mdatp, and re-enables fapolicyd.</t>
+          <t>VMware vSphere 8.0 ESXi STIG remediation playbook. Validates vCenter connectivity, discovers ESXi hosts by hostname list or cluster, loads production STIG config from a YAML file, then applies security, logging, services, and reporting roles. Supports both individual host and cluster-wide targeting.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/mde_gcc/mde_gcc_install.sh, files/mde_gcc/MicrosoftDefenderATPOnboardingLinuxServer.py</t>
+          <t>Yes — Roles: roles/vsphere_stig_security/, roles/vsphere_stig_logging/, roles/vsphere_stig_services/, roles/vsphere_stig_reporting/; File: config/production_stig_config.yml</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>mde_rhel_install.yml</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Full MDE installation on RHEL: installs yum-utils, stops fapolicyd, copies and runs the onboarding Python script, backs up the onboarding JSON, executes the installer shell script with install/monitor/accept flags, then restarts fapolicyd.</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Yes — Files: files/mde/mde_installer-AV-active-S9.4.sh, files/mde/MicrosoftDefenderATPOnboardingLinuxServer.py</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Defender for Endpoint (MDE)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>mde_rhel_health_check.yml</t>
+          <t>mde_gcc_install.yml</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Post-install MDE health validation: checks org_id, healthy status, real-time protection (expects true), and connectivity test (expects ≥10 OK endpoints), asserting each against expected values.</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Installs Microsoft Defender for Endpoint on RHEL (GCC environment variant). Installs yum-utils, stops fapolicyd if present, copies the GCC onboarding script, runs the Python onboarding, restarts mdatp, and re-enables fapolicyd.</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Files: files/mde_gcc/mde_gcc_install.sh, files/mde_gcc/MicrosoftDefenderATPOnboardingLinuxServer.py</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>mde_rhel_post_install.yml</t>
+          <t>mde_rhel_install.yml</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Similar to the health check but expects real-time protection to be false (passive mode). Used for post-install verification before enabling active protection.</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Full MDE installation on RHEL: installs yum-utils, stops fapolicyd, copies and runs the onboarding Python script, backs up the onboarding JSON, executes the installer shell script, then restarts fapolicyd.</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Files: files/mde/mde_installer-AV-active-S9.4.sh, files/mde/MicrosoftDefenderATPOnboardingLinuxServer.py</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Windows Remote PowerShell Execution (WinRM)</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>mde_rhel_health_check.yml</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Post-install MDE health validation: checks org_id, healthy status, real-time protection (expects true), and connectivity test (expects ≥10 OK endpoints), asserting each against expected values.</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>TLS-fix.yml</t>
+          <t>mde_rhel_post_install.yml</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script on Windows hosts with Action, ActionRemoteFile, ADGroupMember, and DomainName parameters for TLS remediation.</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Similar to the health check but expects real-time protection to be false (passive mode). Used for post-install verification before enabling active protection.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>VMware_Disable_SSH.yml</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Runs a PowerShell script against vCenter(s) to disable SSH on VMware hosts, with email reporting parameters and vCenterList input.</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Windows Remote PowerShell Execution (WinRM)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>get_datastores_75_100_used.yml</t>
+          <t>TLS-fix.yml</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script to report on VMware datastores at 75–100% utilization, with email reporting and vCenterList inputs.</t>
+          <t>Runs a PowerShell script on Windows hosts with Action, ActionRemoteFile, ADGroupMember, and DomainName parameters for TLS remediation.</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>move-win-archived-logs.yml</t>
+          <t>VMware_Disable_SSH.yml</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script to move archived Windows logs to a file share target, accepting Action, ADGroupMember, FileShareTarget, and DomainName parameters.</t>
+          <t>Runs a PowerShell script against vCenter(s) to disable SSH on VMware hosts, with email reporting and vCenterList input.</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>remove-OldFiles-UNCPath.yml</t>
+          <t>get_datastores_75_100_used.yml</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script to remove old files from a UNC share path, parameterized with UNC_SharePath, OlderThanDays, and WhatIf (dry-run toggle).</t>
+          <t>Runs a PowerShell script to report on VMware datastores at 75–100% utilization, with email reporting and vCenterList inputs.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>servers_diskclean.yml</t>
+          <t>move-win-archived-logs.yml</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell disk cleanup script on Windows servers with parameters for target folder, included folders, force enable, number of days, filter criteria, AD group, and domain.</t>
+          <t>Runs a PowerShell script to move archived Windows logs to a file share target.</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>servers_pending_reboot_report.yml</t>
+          <t>remove-OldFiles-UNCPath.yml</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script that queries AD group members for pending reboot status and sends an email report.</t>
+          <t>Runs a PowerShell script to remove old files from a UNC share path, with WhatIf dry-run toggle.</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>servers_reboot.yml</t>
+          <t>servers_diskclean.yml</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script to reboot Windows servers from an AD group with configurable delay between reboots and email reporting.</t>
+          <t>Runs a PowerShell disk cleanup script on Windows servers with folder, filter, and age parameters.</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>servers_reboot_report-ByCN.yml</t>
+          <t>servers_pending_reboot_report.yml</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Same as the reboot report but filters by Security Group CN (Common Name) instead of ADGroupMember.</t>
+          <t>Runs a PowerShell script that queries AD group members for pending reboot status and sends an email report.</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>service_accounts_report.yml</t>
+          <t>servers_reboot.yml</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Runs a PowerShell script to report on service account expirations from a specified AD OU path, with email delivery.</t>
+          <t>Runs a PowerShell script to reboot Windows servers from an AD group with configurable delay between reboots and email reporting.</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}} (PowerShell script folder/file supplied at runtime)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Cisco Network — Image Staging</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>servers_reboot_report-ByCN.yml</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Same as the reboot report but filters by Security Group CN instead of ADGroupMember.</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>staging.yml</t>
+          <t>service_accounts_report.yml</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Stages a firmware image to Cisco Cat8000v routers: enables SCP, fetches the image from a backup server to the execution environment, copies it to bootflash via net_put, and verifies the SHA512 hash.</t>
+          <t>Runs a PowerShell script to report on service account expirations from a specified AD OU path, with email delivery.</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Yes — External file: ~/upgrades/{{new_image}} on backup-server (fetched at runtime via SCP)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>staging (1).yml</t>
+          <t>admin_accounts_report.yml</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Identical staging pattern for Cisco Catalyst 9000v switches (Cat9kv).</t>
+          <t>Runs a PowerShell script to report on admin accounts from a specified AD OU path, with email delivery and debug output.</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Yes — External file: ~/upgrades/{{new_image}} on backup-server (fetched at runtime via SCP)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>staging (2).yml</t>
+          <t>admin_accounts_report-v2.yml</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Stages firmware to Nexus 9000v switches: extends VTY exec-timeout, enables SCP server, pulls the image via nxos_file_copy with SCP from a remote server through a specified VRF, resets the connection, and verifies SHA512.</t>
+          <t>V2 of the admin accounts report. Writes a DomainOUs JSON file to the target before executing the PowerShell script, supporting multi-domain OU input.</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Yes — External file: {{remote_file}} on {{remote_scp_server}} (pulled at runtime via SCP)</t>
+          <t>Yes — Files: files/{{var_ps_folder}}/{{var_ps_script_file}}</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>staging-with-scp.yml</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Enhanced N9kv staging with comprehensive pre-flight checks: validates variables, tests TCP/22 connectivity, verifies bootflash free space against expected file size + 10% buffer, performs SCP copy, verifies file size match, calculates SHA512 hash, then restores VTY timeout and disables SCP server.</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Yes — External file: {{remote_file}} on {{remote_scp_server}} (pulled at runtime via SCP)</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Windows File Operations (AD-Driven / Inline PS)</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Cisco Network — Upgrades</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>file-deletion_with-UNCPath_AD-Group.yml</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Queries AD for computer objects in a security group, builds a dynamic inventory, then deletes files older than N days from UNC paths on each server using an inline PowerShell function.</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>No — Inline PowerShell; AD group DN and parameters supplied at runtime</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>upgrade.yml</t>
+          <t>file-move_with-UNCPath_AD-Group.yml</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Upgrades Cisco Cat8000v: extracts version from the image filename, changes the boot system, renames the old packages.conf, runs install add file ... activate commit, waits for reboot, and asserts the new version.</t>
+          <t>Queries AD for computer objects in a security group, builds a dynamic inventory, then moves files older than N days from UNC source paths to a target share using an inline PowerShell function.</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>No — Assumes {{new_image}} is already staged in bootflash</t>
+          <t>No — Inline PowerShell; AD group DN and parameters supplied at runtime</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>upgrade (1).yml</t>
+          <t>file-move_with-UNCPath_AD-Group-TEST.yml</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Same upgrade workflow for Catalyst 9000v (Cat9kv) switches.</t>
+          <t>Test variant of UNC file move. Adds explicit AD credential handling (PSCredential) for environments requiring authenticated AD queries. Same move logic as the production version.</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>No — Assumes {{new_image}} is already staged in bootflash</t>
+          <t>No — Inline PowerShell; AD group DN and parameters supplied at runtime</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>upgrade (2).yml</t>
+          <t>file-move_with-UNCPath_AD-Group-TEST(1).yml</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Upgrades Nexus 9000v switches using nxos_install_os, waits for reboot, resets SSH, and asserts the post-upgrade version.</t>
+          <t>Second test variant of UNC file move. Uses -Server parameter for cross-domain AD queries (specifies DomainName). Same core move logic.</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>No — Assumes {{new_image}} is already staged in bootflash</t>
+          <t>No — Inline PowerShell; AD group DN and parameters supplied at runtime</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>upgrade_64.yml</t>
+          <t>file-move_with-LocalPath_AD-Group.yml</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Upgrades Nexus 9000v switches running the 64-bit NX-OS image (nxos64-cs), using the same nxos_install_os workflow but parsing the 64-bit image filename convention.</t>
+          <t>Queries AD for computer objects in a security group, builds a dynamic inventory, then moves files from local paths on each server to a target share using a two-play design (inventory build, then execute on dynamic group).</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>No — Assumes {{new_image}} is already staged in bootflash</t>
+          <t>No — Inline PowerShell; AD group DN and parameters supplied at runtime</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Cisco Network — Other</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>file-move_with-LocalPath_Inventory.yml</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Moves archived log files from a local source path to a share target on Windows hosts from the static inventory (no AD lookup). Uses an inline PowerShell Move-files function.</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>No — Inline PowerShell; source_path, target_path, file_filter, days_old supplied at runtime</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>nexus_password_change.yml</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Changes the admin password on Cisco Nexus switches. Constructs a password from a prefix + hostname + suffix, applies it, saves config, resets the connection, and verifies by reconnecting with the new credentials.</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Cisco Network — Image Staging</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>set_user_key.yml</t>
+          <t>staging.yml</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Creates a local user account on Nexus 9000 switches with an SSH public key and a specified role, then saves the configuration.</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>No — SSH public key is passed via the {{ssh_key}} variable</t>
+          <t>Stages firmware to Cisco Cat8000v routers: enables SCP, fetches image from backup server, copies to bootflash via net_put, verifies SHA512 hash.</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Yes — External file: ~/upgrades/{{new_image}} on backup-server</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>show_discovery.yml</t>
+          <t>staging (1).yml / staging (4).yml</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Runs 'show cdp neighbor detail' and 'show vpc' on Nexus switches for network discovery/documentation.</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Identical staging pattern for Cisco Catalyst 9000v (Cat9kv) switches.</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Yes — External file: ~/upgrades/{{new_image}} on backup-server</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Linux Administration</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>staging (2).yml / staging (5).yml</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Stages firmware to Nexus 9000v: extends VTY timeout, enables SCP server, pulls image via nxos_file_copy through a VRF, resets connection, verifies SHA512.</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Yes — External file: {{remote_file}} on {{remote_scp_server}}</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>dnf_update.yml</t>
+          <t>staging-with-scp.yml</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Runs 'dnf upgrade -y' on all targeted Linux hosts (simple package update).</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Enhanced N9kv staging with pre-flight checks: validates variables, tests TCP/22, verifies bootflash space, performs SCP copy, verifies file size + SHA512, then restores timeout and disables SCP.</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Yes — External file: {{remote_file}} on {{remote_scp_server}}</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>firewall_rich_rule.yml</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Configures RHEL 9 firewalld to restrict a service (default SSH) to specific IP addresses/subnets via rich rules. Includes input validation, admin-IP safety check before removing the broad service/port, and verification output.</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Cisco Network — Upgrades</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>rhel_change_root_pw.yml</t>
+          <t>upgrade.yml</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Enterprise-grade RHEL password change playbook for AAP 2.5 surveys. Features password complexity validation, password confirmation, self-lockout protection, shadow file backup with scheduled cleanup, SHA512 hashing, password aging policy, audit logging, and emergency rollback on failure.</t>
+          <t>Upgrades Cisco Cat8000v: changes boot system, renames old packages.conf, runs install add file activate commit, waits for reboot, asserts new version.</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No — Assumes {{new_image}} already staged in bootflash</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>registry_to_satellite.yml</t>
+          <t>upgrade (1).yml / upgrade (4).yml</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Registers RHEL 9 systems with Red Hat Satellite/Foreman: unregisters and cleans existing subscriptions, cleans DNF/YUM caches, builds a registration URL with activation key and org/location/hostgroup IDs, calls the Satellite registration API via curl, and verifies repositories are available.</t>
+          <t>Same upgrade workflow for Catalyst 9000v (Cat9kv) switches.</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No — Assumes {{new_image}} already staged in bootflash</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>setup-ansible-vROPS-user.yml</t>
+          <t>upgrade (2).yml / upgrade (5).yml</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Creates an Ansible service account on Linux hosts (designed for vROps targets): creates user/group, adds to wheel, deploys an SSH public key, configures passwordless sudo, and ensures SSHD is running.</t>
+          <t>Upgrades Nexus 9000v using nxos_install_os, waits for reboot, resets SSH, asserts post-upgrade version.</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>No — SSH public key is passed via the {{var_pub_key}} variable</t>
+          <t>No — Assumes {{new_image}} already staged in bootflash</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>VMware Operations</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>upgrade_64.yml</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Upgrades Nexus 9000v running 64-bit NX-OS (nxos64-cs), same nxos_install_os workflow but parses 64-bit filename convention.</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>No — Assumes {{new_image}} already staged in bootflash</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>vm_remove_snapshot.yml</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Removes VM snapshots by applying a vm_snapshot role with vCenter credentials passed as variables.</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>Yes — Role: roles/vm_snapshot/</t>
-        </is>
-      </c>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Cisco Network — Configuration Management</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Network / Connectivity Testing</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>backup.yml</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Backs up running configs of Cisco network devices (N9kv/Cat9k) to a GitLab/Gitea repository in a timestamped branch via ansible.scm. Then dynamically creates AAP job templates for Diff and Restore playbooks with branch-selection surveys.</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Companion playbooks: diff.yml, restore.yml; requires GitLab/Gitea repo and AAP controller access</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>vm_port-test_TCP22.yml</t>
+          <t>diff.yml</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Tests TCP port 22 (SSH) connectivity from the Ansible host to a list of VMs/hosts with a 1-second timeout per host.</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Compares running Nexus 9000 configurations against a saved config in a GitLab/Gitea branch using nxos_config diff_against: intended. Used by the backup.yml-generated job template.</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Yes — External: Git repo at {{git_url}} (config files in network_backup_files/)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
+          <t>restore.yml</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Restores Nexus 9000 configurations from a GitLab/Gitea branch. Copies saved config to bootflash, runs configure replace, then cleans up the temp file.</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Yes — External: Git repo at {{git_url}} (config files in network_backup_files/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>command.yml</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Runs an arbitrary Cisco NX-OS command (passed via {{var_command}}) on targeted switches. Generic utility playbook.</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Cisco Network — Other</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>nexus_password_change.yml</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Changes the admin password on Cisco Nexus switches. Constructs password from prefix + hostname + suffix, applies, saves, resets connection, verifies.</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>set_user_key.yml</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Creates a local user account on Nexus 9000 switches with an SSH public key and role, saves config.</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>No — SSH key passed via {{ssh_key}} variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>show_discovery.yml</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Runs 'show cdp neighbor detail' and 'show vpc' on Nexus switches for network discovery.</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>create_snmp_account.yml</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Configures an SNMPv3 user on Cisco Nexus 9K switches with auth (SHA/MD5) and privacy (AES/DES) protocols. Validates inputs, applies config, verifies, and optionally sets contact/location.</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Linux Administration</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>dnf_update.yml</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Runs 'dnf upgrade -y' on all targeted Linux hosts.</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>firewall_rich_rule.yml</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Configures RHEL 9 firewalld to restrict a service to specific IPs/subnets via rich rules, with input validation and admin-IP safety checks.</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>rhel_change_root_pw.yml</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise-grade RHEL password change for AAP 2.5 surveys. Password complexity validation, self-lockout protection, shadow backup, SHA512 hashing, aging policy, audit logging, emergency rollback.</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>registry_to_satellite.yml</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Registers RHEL 9 systems with Red Hat Satellite/Foreman: unregisters, cleans caches, calls registration API with activation key, verifies repositories.</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>setup-ansible-vROPS-user.yml</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Creates an Ansible service account on Linux hosts: user/group, wheel membership, SSH public key, passwordless sudo, ensures SSHD running.</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>No — SSH key passed via {{var_pub_key}} variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>create_RHEL_local.yml</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Creates a local user account on RHEL hosts with a password (SHA512 hashed), adds to wheel group. Simpler than the password-change playbook — no complexity validation or backup.</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>account_password_update.yml</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Resets an Active Directory account password using the microsoft.ad collection and AAP controller integration. Delegates to the 'account' role.</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Role: roles/account/; Collections: microsoft.ad, ansible.controller</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>aria_operations_firewall.yml</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Comprehensive VMware Aria 8.18 iptables firewall hardening. Backs up rules, removes blanket ACCEPT/REJECT rules from INPUT/TCP/UDP chains, adds cluster-node allow rules, adds per-port allow rules for specified networks/IPs, adds catch-all DROP to TCP/UDP chains, persists via systemd service + rc.local + cron @reboot.</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>VMware Operations</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>vm_remove_snapshot.yml</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Removes VM snapshots by applying a vm_snapshot role with vCenter credentials.</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Role: roles/vm_snapshot/</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>esxi_port_test.yml</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Dynamically discovers ESXi hosts in specified vCenter clusters via community.vmware, then runs port connectivity tests against them using an included task file.</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Yes — Task file: tasks/get_esxi_inventory.yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Network / Connectivity Testing</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n"/>
+      <c r="C71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>vm_port-test_TCP22.yml</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Tests TCP port 22 connectivity from the Ansible host to a list of VMs/hosts with a 1-second timeout.</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
           <t>vm_port_test.yml</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>General multi-port connectivity test: iterates over a list of VMs and checks multiple ports (e.g., 22, 443, 80) by including an external tasks file.</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>General multi-port connectivity test: iterates over VMs and checks multiple ports via an external tasks file.</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Yes — Task file: tasks/ports_check.yml</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>PowerFlex Manager API</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>pf_check_managed_resources.yml</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Queries the PowerFlex Manager API for deployed services and managed/unmanaged resource groups. Generates a detailed report indicating whether actual host password updates are supported (deployed/managed) or only credential-store updates (discovered/unmanaged).</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>pf_list_all_cred_types.yml</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Queries the PowerFlex Manager API and lists all unique credential type names (e.g., OSCredential, ServerCredential). Used to discover correct API type names for filtering in credential update playbooks.</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>pf_credential_update.yml</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Updates credentials in the PowerFlex Manager credential store by name pattern. Authenticates via REST API, fetches all credentials, filters by include/exclude name patterns and optional type filter, supports dry-run mode. Update PUT calls are commented out (ready to enable).</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>pf_update_credentials_by_label.yml</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Updates credentials in the PowerFlex Manager credential store by exact label match. Fetches credentials by label via API filtering, supports type filtering and dry-run mode. Includes active PUT calls for live updates (XML body format).</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>Zabbix API</t>
         </is>
       </c>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="B79" s="2" t="n"/>
+      <c r="C79" s="2" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>zab_token_renewal.yml</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>Extends the expiration of Zabbix user API tokens. Authenticates to the Zabbix JSON-RPC API, looks up the target user and their tokens (optionally filtered by token name), calculates a new expiration based on days/months/years/never-expire inputs, updates the token(s), displays a summary, and logs out.</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Extends Zabbix user API token expiration. Authenticates to JSON-RPC API, looks up user/tokens, calculates new expiration from days/months/years/never-expire, updates tokens, displays summary, logs out.</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C54"/>
+  <autoFilter ref="A1:C80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>